<commit_message>
Add hero block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 38
</commit_message>
<xml_diff>
--- a/tools/importer/reports/commerce-import.report.xlsx
+++ b/tools/importer/reports/commerce-import.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="162">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,6 +40,30 @@
     <t>url</t>
   </si>
   <si>
+    <t>accessories.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>accessories</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>PLP Template</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:18.096Z</t>
+  </si>
+  <si>
+    <t>Accessories</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/accessories</t>
+  </si>
+  <si>
     <t>business.report.json</t>
   </si>
   <si>
@@ -49,12 +73,6 @@
     <t>business</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>landing-page</t>
   </si>
   <si>
@@ -73,10 +91,7 @@
     <t>coffee</t>
   </si>
   <si>
-    <t>PLP Template</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:27:50.439Z</t>
+    <t>2026-10-08T01:49:50.301Z</t>
   </si>
   <si>
     <t>Frescopa Coffee</t>
@@ -145,7 +160,7 @@
     <t>en/coffee</t>
   </si>
   <si>
-    <t>2026-10-08T01:27:57.808Z</t>
+    <t>2026-10-08T01:49:55.677Z</t>
   </si>
   <si>
     <t>https://frescopa.coffee/en/coffee</t>
@@ -178,6 +193,36 @@
     <t>https://frescopa.coffee/en/subscription</t>
   </si>
   <si>
+    <t>en/tea.report.json</t>
+  </si>
+  <si>
+    <t>en/tea</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:22.279Z</t>
+  </si>
+  <si>
+    <t>Tea</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/en/tea</t>
+  </si>
+  <si>
+    <t>es/accessories.report.json</t>
+  </si>
+  <si>
+    <t>es/accessories</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:26.375Z</t>
+  </si>
+  <si>
+    <t>Accesorios</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/es/accessories</t>
+  </si>
+  <si>
     <t>es/business.report.json</t>
   </si>
   <si>
@@ -199,7 +244,7 @@
     <t>es/coffee</t>
   </si>
   <si>
-    <t>2026-10-08T01:28:05.457Z</t>
+    <t>2026-10-08T01:50:01.434Z</t>
   </si>
   <si>
     <t>Café Frescopa</t>
@@ -238,6 +283,36 @@
     <t>https://frescopa.coffee/es/subscription</t>
   </si>
   <si>
+    <t>es/tea.report.json</t>
+  </si>
+  <si>
+    <t>es/tea</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:30.736Z</t>
+  </si>
+  <si>
+    <t>Té</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/es/tea</t>
+  </si>
+  <si>
+    <t>fr/accessories.report.json</t>
+  </si>
+  <si>
+    <t>fr/accessories</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:35.876Z</t>
+  </si>
+  <si>
+    <t>Accessoires</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/fr/accessories</t>
+  </si>
+  <si>
     <t>fr/business.report.json</t>
   </si>
   <si>
@@ -259,7 +334,7 @@
     <t>fr/coffee</t>
   </si>
   <si>
-    <t>2026-10-08T01:28:12.265Z</t>
+    <t>2026-10-08T01:50:06.587Z</t>
   </si>
   <si>
     <t>https://frescopa.coffee/fr/coffee</t>
@@ -295,6 +370,36 @@
     <t>https://frescopa.coffee/fr/subscription</t>
   </si>
   <si>
+    <t>fr/tea.report.json</t>
+  </si>
+  <si>
+    <t>fr/tea</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:40.449Z</t>
+  </si>
+  <si>
+    <t>Thé</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/fr/tea</t>
+  </si>
+  <si>
+    <t>jp/accessories.report.json</t>
+  </si>
+  <si>
+    <t>jp/accessories</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:44.131Z</t>
+  </si>
+  <si>
+    <t>小物</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/jp/accessories</t>
+  </si>
+  <si>
     <t>jp/business.report.json</t>
   </si>
   <si>
@@ -316,7 +421,7 @@
     <t>jp/coffee</t>
   </si>
   <si>
-    <t>2026-10-08T01:28:18.510Z</t>
+    <t>2026-10-08T01:50:12.631Z</t>
   </si>
   <si>
     <t>フレスコパコーヒー</t>
@@ -353,6 +458,21 @@
   </si>
   <si>
     <t>https://frescopa.coffee/jp/subscription</t>
+  </si>
+  <si>
+    <t>jp/tea.report.json</t>
+  </si>
+  <si>
+    <t>jp/tea</t>
+  </si>
+  <si>
+    <t>2026-10-08T01:50:47.890Z</t>
+  </si>
+  <si>
+    <t>茶</t>
+  </si>
+  <si>
+    <t>https://frescopa.coffee/jp/tea</t>
   </si>
   <si>
     <t>experiments/value-prop-headline-test/challenger-1.report.json</t>
@@ -765,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -815,40 +935,40 @@
       <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>12</v>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
       </c>
-      <c r="D3">
-        <v>2</v>
+      <c r="D3" t="s">
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
         <v>20</v>
@@ -868,103 +988,103 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>27</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>28</v>
-      </c>
-      <c r="I4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>33</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>34</v>
-      </c>
-      <c r="I5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
         <v>36</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>37</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
         <v>38</v>
       </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>39</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>40</v>
-      </c>
-      <c r="I6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
         <v>42</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
       </c>
       <c r="C7" t="s">
         <v>43</v>
       </c>
-      <c r="D7">
-        <v>2</v>
+      <c r="D7" t="s">
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F7" t="s">
         <v>20</v>
@@ -973,36 +1093,36 @@
         <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="D8" t="s">
-        <v>12</v>
+      <c r="D8">
+        <v>2</v>
       </c>
       <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
         <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
       </c>
       <c r="G8" t="s">
         <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I8" t="s">
         <v>50</v>
@@ -1013,54 +1133,54 @@
         <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="I10" t="s">
         <v>59</v>
@@ -1071,19 +1191,19 @@
         <v>60</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
         <v>61</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
         <v>13</v>
-      </c>
-      <c r="F11" t="s">
-        <v>20</v>
       </c>
       <c r="G11" t="s">
         <v>62</v>
@@ -1100,19 +1220,19 @@
         <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>66</v>
       </c>
-      <c r="D12" t="s">
-        <v>12</v>
+      <c r="D12">
+        <v>1</v>
       </c>
       <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
         <v>13</v>
-      </c>
-      <c r="F12" t="s">
-        <v>14</v>
       </c>
       <c r="G12" t="s">
         <v>67</v>
@@ -1129,19 +1249,19 @@
         <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="C13" t="s">
         <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G13" t="s">
         <v>72</v>
@@ -1163,14 +1283,14 @@
       <c r="C14" t="s">
         <v>76</v>
       </c>
-      <c r="D14" t="s">
-        <v>12</v>
+      <c r="D14">
+        <v>2</v>
       </c>
       <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
         <v>13</v>
-      </c>
-      <c r="F14" t="s">
-        <v>14</v>
       </c>
       <c r="G14" t="s">
         <v>77</v>
@@ -1187,16 +1307,16 @@
         <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="C15" t="s">
         <v>81</v>
       </c>
-      <c r="D15">
-        <v>2</v>
+      <c r="D15" t="s">
+        <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" t="s">
         <v>20</v>
@@ -1205,152 +1325,152 @@
         <v>82</v>
       </c>
       <c r="H15" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="I15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F16" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
+        <v>91</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
       </c>
       <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
         <v>13</v>
       </c>
-      <c r="F17" t="s">
-        <v>14</v>
-      </c>
       <c r="G17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I17" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" t="s">
-        <v>12</v>
+        <v>96</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
       </c>
       <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
         <v>13</v>
       </c>
-      <c r="F18" t="s">
-        <v>14</v>
-      </c>
       <c r="G18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
-      </c>
-      <c r="D19">
-        <v>2</v>
+        <v>101</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F19" t="s">
         <v>20</v>
       </c>
       <c r="G19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>105</v>
-      </c>
-      <c r="D20" t="s">
-        <v>12</v>
+        <v>106</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
       </c>
       <c r="E20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
         <v>13</v>
       </c>
-      <c r="F20" t="s">
-        <v>14</v>
-      </c>
       <c r="G20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="I20" t="s">
         <v>108</v>
@@ -1361,19 +1481,19 @@
         <v>109</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
         <v>110</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F21" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G21" t="s">
         <v>111</v>
@@ -1390,57 +1510,289 @@
         <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C22" t="s">
         <v>115</v>
       </c>
       <c r="D22" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G22" t="s">
         <v>116</v>
       </c>
       <c r="H22" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="I22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D23" t="s">
-        <v>12</v>
+        <v>120</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
       </c>
       <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" t="s">
         <v>13</v>
       </c>
-      <c r="F23" t="s">
-        <v>14</v>
-      </c>
       <c r="G23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H23" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="I23" t="s">
-        <v>121</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
+        <v>126</v>
+      </c>
+      <c r="H24" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" t="s">
+        <v>20</v>
+      </c>
+      <c r="G25" t="s">
+        <v>131</v>
+      </c>
+      <c r="H25" t="s">
+        <v>132</v>
+      </c>
+      <c r="I25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>135</v>
+      </c>
+      <c r="D26">
+        <v>2</v>
+      </c>
+      <c r="E26" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" t="s">
+        <v>136</v>
+      </c>
+      <c r="H26" t="s">
+        <v>137</v>
+      </c>
+      <c r="I26" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>139</v>
+      </c>
+      <c r="B27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27" t="s">
+        <v>141</v>
+      </c>
+      <c r="H27" t="s">
+        <v>142</v>
+      </c>
+      <c r="I27" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>144</v>
+      </c>
+      <c r="B28" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" t="s">
+        <v>145</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" t="s">
+        <v>146</v>
+      </c>
+      <c r="H28" t="s">
+        <v>147</v>
+      </c>
+      <c r="I28" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>149</v>
+      </c>
+      <c r="B29" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" t="s">
+        <v>150</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" t="s">
+        <v>151</v>
+      </c>
+      <c r="H29" t="s">
+        <v>152</v>
+      </c>
+      <c r="I29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" t="s">
+        <v>155</v>
+      </c>
+      <c r="D30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" t="s">
+        <v>20</v>
+      </c>
+      <c r="G30" t="s">
+        <v>156</v>
+      </c>
+      <c r="H30" t="s">
+        <v>39</v>
+      </c>
+      <c r="I30" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>158</v>
+      </c>
+      <c r="B31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" t="s">
+        <v>160</v>
+      </c>
+      <c r="H31" t="s">
+        <v>83</v>
+      </c>
+      <c r="I31" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>